<commit_message>
Fix tip-section volume calculation: treat treetop section as a cone rather than a frustum
</commit_message>
<xml_diff>
--- a/outputs/resultado_final_REFERENCIA_python.xlsx
+++ b/outputs/resultado_final_REFERENCIA_python.xlsx
@@ -409,16 +409,16 @@
         <v>23.3</v>
       </c>
       <c r="D2">
-        <v>0.163</v>
+        <v>0.1622</v>
       </c>
       <c r="E2">
-        <v>0.1617</v>
+        <v>0.1621</v>
       </c>
       <c r="F2">
         <v>0.1622</v>
       </c>
       <c r="G2">
-        <v>0.5286</v>
+        <v>0.5262</v>
       </c>
       <c r="H2">
         <v>0.912</v>
@@ -435,16 +435,16 @@
         <v>26.4</v>
       </c>
       <c r="D3">
-        <v>0.2783</v>
+        <v>0.2776</v>
       </c>
       <c r="E3">
-        <v>0.2771</v>
+        <v>0.2775</v>
       </c>
       <c r="F3">
         <v>0.2775</v>
       </c>
       <c r="G3">
-        <v>0.4733</v>
+        <v>0.4722</v>
       </c>
       <c r="H3">
         <v>0.9163</v>
@@ -461,16 +461,16 @@
         <v>27.7</v>
       </c>
       <c r="D4">
-        <v>0.37</v>
+        <v>0.3693</v>
       </c>
       <c r="E4">
-        <v>0.3687</v>
+        <v>0.3691</v>
       </c>
       <c r="F4">
         <v>0.3691</v>
       </c>
       <c r="G4">
-        <v>0.4843</v>
+        <v>0.4833</v>
       </c>
       <c r="H4">
         <v>0.9018</v>
@@ -487,16 +487,16 @@
         <v>21.3</v>
       </c>
       <c r="D5">
-        <v>0.1182</v>
+        <v>0.1175</v>
       </c>
       <c r="E5">
-        <v>0.117</v>
+        <v>0.1174</v>
       </c>
       <c r="F5">
         <v>0.1174</v>
       </c>
       <c r="G5">
-        <v>0.4864</v>
+        <v>0.4836</v>
       </c>
       <c r="H5">
         <v>0.8813</v>
@@ -513,16 +513,16 @@
         <v>27.2</v>
       </c>
       <c r="D6">
-        <v>0.2603</v>
+        <v>0.2597</v>
       </c>
       <c r="E6">
-        <v>0.2593</v>
+        <v>0.2596</v>
       </c>
       <c r="F6">
         <v>0.2596</v>
       </c>
       <c r="G6">
-        <v>0.4974</v>
+        <v>0.4964</v>
       </c>
       <c r="H6">
         <v>0.9099</v>
@@ -539,16 +539,16 @@
         <v>28.5</v>
       </c>
       <c r="D7">
-        <v>0.3353</v>
+        <v>0.3346</v>
       </c>
       <c r="E7">
-        <v>0.334</v>
+        <v>0.3344</v>
       </c>
       <c r="F7">
         <v>0.3344</v>
       </c>
       <c r="G7">
-        <v>0.4597</v>
+        <v>0.4588</v>
       </c>
       <c r="H7">
         <v>0.8609</v>
@@ -565,16 +565,16 @@
         <v>28.3</v>
       </c>
       <c r="D8">
-        <v>0.327</v>
+        <v>0.3263</v>
       </c>
       <c r="E8">
-        <v>0.3258</v>
+        <v>0.3261</v>
       </c>
       <c r="F8">
         <v>0.3262</v>
       </c>
       <c r="G8">
-        <v>0.4566</v>
+        <v>0.4557</v>
       </c>
       <c r="H8">
         <v>0.8875</v>
@@ -591,16 +591,16 @@
         <v>27.1</v>
       </c>
       <c r="D9">
-        <v>0.2486</v>
+        <v>0.248</v>
       </c>
       <c r="E9">
-        <v>0.2475</v>
+        <v>0.2478</v>
       </c>
       <c r="F9">
         <v>0.2479</v>
       </c>
       <c r="G9">
-        <v>0.4684</v>
+        <v>0.4673</v>
       </c>
       <c r="H9">
         <v>0.8814</v>
@@ -617,16 +617,16 @@
         <v>27</v>
       </c>
       <c r="D10">
-        <v>0.2505</v>
+        <v>0.2498</v>
       </c>
       <c r="E10">
-        <v>0.2494</v>
+        <v>0.2497</v>
       </c>
       <c r="F10">
         <v>0.2497</v>
       </c>
       <c r="G10">
-        <v>0.4338</v>
+        <v>0.4328</v>
       </c>
       <c r="H10">
         <v>0.8538</v>
@@ -643,16 +643,16 @@
         <v>27.2</v>
       </c>
       <c r="D11">
-        <v>0.2703</v>
+        <v>0.2697</v>
       </c>
       <c r="E11">
-        <v>0.2692</v>
+        <v>0.2695</v>
       </c>
       <c r="F11">
         <v>0.2696</v>
       </c>
       <c r="G11">
-        <v>0.4457</v>
+        <v>0.4447</v>
       </c>
       <c r="H11">
         <v>0.8819</v>
@@ -669,16 +669,16 @@
         <v>27.4</v>
       </c>
       <c r="D12">
-        <v>0.2757</v>
+        <v>0.2751</v>
       </c>
       <c r="E12">
-        <v>0.2747</v>
+        <v>0.275</v>
       </c>
       <c r="F12">
         <v>0.275</v>
       </c>
       <c r="G12">
-        <v>0.4655</v>
+        <v>0.4645</v>
       </c>
       <c r="H12">
         <v>0.9005</v>
@@ -695,16 +695,16 @@
         <v>28</v>
       </c>
       <c r="D13">
-        <v>0.3333</v>
+        <v>0.3328</v>
       </c>
       <c r="E13">
-        <v>0.3323</v>
+        <v>0.3326</v>
       </c>
       <c r="F13">
         <v>0.3326</v>
       </c>
       <c r="G13">
-        <v>0.4866</v>
+        <v>0.4857</v>
       </c>
       <c r="H13">
         <v>0.9208</v>
@@ -721,16 +721,16 @@
         <v>28</v>
       </c>
       <c r="D14">
-        <v>0.3321</v>
+        <v>0.3315</v>
       </c>
       <c r="E14">
-        <v>0.331</v>
+        <v>0.3313</v>
       </c>
       <c r="F14">
         <v>0.3313</v>
       </c>
       <c r="G14">
-        <v>0.4515</v>
+        <v>0.4506</v>
       </c>
       <c r="H14">
         <v>0.8895999999999999</v>
@@ -747,16 +747,16 @@
         <v>24.9</v>
       </c>
       <c r="D15">
-        <v>0.1675</v>
+        <v>0.1668</v>
       </c>
       <c r="E15">
-        <v>0.1663</v>
+        <v>0.1667</v>
       </c>
       <c r="F15">
         <v>0.1667</v>
       </c>
       <c r="G15">
-        <v>0.4879</v>
+        <v>0.4857</v>
       </c>
       <c r="H15">
         <v>0.8972</v>
@@ -773,16 +773,16 @@
         <v>26.8</v>
       </c>
       <c r="D16">
-        <v>0.212</v>
+        <v>0.2114</v>
       </c>
       <c r="E16">
-        <v>0.2109</v>
+        <v>0.2112</v>
       </c>
       <c r="F16">
         <v>0.2113</v>
       </c>
       <c r="G16">
-        <v>0.4926</v>
+        <v>0.4911</v>
       </c>
       <c r="H16">
         <v>0.8993</v>
@@ -799,16 +799,16 @@
         <v>26.3</v>
       </c>
       <c r="D17">
-        <v>0.2098</v>
+        <v>0.2092</v>
       </c>
       <c r="E17">
-        <v>0.2088</v>
+        <v>0.2091</v>
       </c>
       <c r="F17">
         <v>0.2091</v>
       </c>
       <c r="G17">
-        <v>0.4932</v>
+        <v>0.4918</v>
       </c>
       <c r="H17">
         <v>0.9073</v>
@@ -825,16 +825,16 @@
         <v>28.5</v>
       </c>
       <c r="D18">
-        <v>0.3031</v>
+        <v>0.3024</v>
       </c>
       <c r="E18">
-        <v>0.3019</v>
+        <v>0.3022</v>
       </c>
       <c r="F18">
         <v>0.3023</v>
       </c>
       <c r="G18">
-        <v>0.4769</v>
+        <v>0.4758</v>
       </c>
       <c r="H18">
         <v>0.9086</v>
@@ -851,16 +851,16 @@
         <v>25.7</v>
       </c>
       <c r="D19">
-        <v>0.187</v>
+        <v>0.1864</v>
       </c>
       <c r="E19">
-        <v>0.1859</v>
+        <v>0.1862</v>
       </c>
       <c r="F19">
         <v>0.1863</v>
       </c>
       <c r="G19">
-        <v>0.4741</v>
+        <v>0.4724</v>
       </c>
       <c r="H19">
         <v>0.887</v>
@@ -877,16 +877,16 @@
         <v>27</v>
       </c>
       <c r="D20">
-        <v>0.2276</v>
+        <v>0.227</v>
       </c>
       <c r="E20">
-        <v>0.2265</v>
+        <v>0.2268</v>
       </c>
       <c r="F20">
         <v>0.2269</v>
       </c>
       <c r="G20">
-        <v>0.4616</v>
+        <v>0.4602</v>
       </c>
       <c r="H20">
         <v>0.8859</v>
@@ -903,16 +903,16 @@
         <v>28.2</v>
       </c>
       <c r="D21">
-        <v>0.309</v>
+        <v>0.3083</v>
       </c>
       <c r="E21">
-        <v>0.3078</v>
+        <v>0.3081</v>
       </c>
       <c r="F21">
         <v>0.3082</v>
       </c>
       <c r="G21">
-        <v>0.4776</v>
+        <v>0.4766</v>
       </c>
       <c r="H21">
         <v>0.9056999999999999</v>
@@ -929,16 +929,16 @@
         <v>25.6</v>
       </c>
       <c r="D22">
-        <v>0.187</v>
+        <v>0.1862</v>
       </c>
       <c r="E22">
-        <v>0.1857</v>
+        <v>0.1861</v>
       </c>
       <c r="F22">
         <v>0.1862</v>
       </c>
       <c r="G22">
-        <v>0.4822</v>
+        <v>0.4801</v>
       </c>
       <c r="H22">
         <v>0.9058</v>
@@ -955,16 +955,16 @@
         <v>27.7</v>
       </c>
       <c r="D23">
-        <v>0.3237</v>
+        <v>0.3231</v>
       </c>
       <c r="E23">
-        <v>0.3226</v>
+        <v>0.3229</v>
       </c>
       <c r="F23">
         <v>0.3229</v>
       </c>
       <c r="G23">
-        <v>0.4803</v>
+        <v>0.4794</v>
       </c>
       <c r="H23">
         <v>0.9125</v>
@@ -981,16 +981,16 @@
         <v>21.3</v>
       </c>
       <c r="D24">
-        <v>0.1091</v>
+        <v>0.1083</v>
       </c>
       <c r="E24">
-        <v>0.1078</v>
+        <v>0.1082</v>
       </c>
       <c r="F24">
         <v>0.1083</v>
       </c>
       <c r="G24">
-        <v>0.5063</v>
+        <v>0.5026</v>
       </c>
       <c r="H24">
         <v>0.8978</v>
@@ -1007,16 +1007,16 @@
         <v>28.4</v>
       </c>
       <c r="D25">
-        <v>0.3883</v>
+        <v>0.3878</v>
       </c>
       <c r="E25">
-        <v>0.3873</v>
+        <v>0.3876</v>
       </c>
       <c r="F25">
         <v>0.3876</v>
       </c>
       <c r="G25">
-        <v>0.4957</v>
+        <v>0.495</v>
       </c>
       <c r="H25">
         <v>0.9146</v>
@@ -1033,16 +1033,16 @@
         <v>22</v>
       </c>
       <c r="D26">
-        <v>0.1091</v>
+        <v>0.1084</v>
       </c>
       <c r="E26">
-        <v>0.1079</v>
+        <v>0.1083</v>
       </c>
       <c r="F26">
         <v>0.1083</v>
       </c>
       <c r="G26">
-        <v>0.4734</v>
+        <v>0.4701</v>
       </c>
       <c r="H26">
         <v>0.8294</v>
@@ -1059,16 +1059,16 @@
         <v>27.1</v>
       </c>
       <c r="D27">
-        <v>0.2808</v>
+        <v>0.2803</v>
       </c>
       <c r="E27">
-        <v>0.2798</v>
+        <v>0.2801</v>
       </c>
       <c r="F27">
         <v>0.2802</v>
       </c>
       <c r="G27">
-        <v>0.5028</v>
+        <v>0.5018</v>
       </c>
       <c r="H27">
         <v>0.916</v>
@@ -1085,16 +1085,16 @@
         <v>27.5</v>
       </c>
       <c r="D28">
-        <v>0.2994</v>
+        <v>0.2988</v>
       </c>
       <c r="E28">
-        <v>0.2983</v>
+        <v>0.2986</v>
       </c>
       <c r="F28">
         <v>0.2986</v>
       </c>
       <c r="G28">
-        <v>0.4825</v>
+        <v>0.4815</v>
       </c>
       <c r="H28">
         <v>0.9044</v>
@@ -1111,16 +1111,16 @@
         <v>13.6</v>
       </c>
       <c r="D29">
-        <v>0.0196</v>
+        <v>0.0184</v>
       </c>
       <c r="E29">
-        <v>0.0177</v>
+        <v>0.0183</v>
       </c>
       <c r="F29">
         <v>0.0184</v>
       </c>
       <c r="G29">
-        <v>0.5775</v>
+        <v>0.5403</v>
       </c>
       <c r="H29">
         <v>0.8289</v>
@@ -1137,16 +1137,16 @@
         <v>14.4</v>
       </c>
       <c r="D30">
-        <v>0.0281</v>
+        <v>0.027</v>
       </c>
       <c r="E30">
-        <v>0.0264</v>
+        <v>0.0269</v>
       </c>
       <c r="F30">
         <v>0.027</v>
       </c>
       <c r="G30">
-        <v>0.5</v>
+        <v>0.4799</v>
       </c>
       <c r="H30">
         <v>0.773</v>
@@ -1163,16 +1163,16 @@
         <v>24.4</v>
       </c>
       <c r="D31">
-        <v>0.1675</v>
+        <v>0.1669</v>
       </c>
       <c r="E31">
-        <v>0.1664</v>
+        <v>0.1668</v>
       </c>
       <c r="F31">
         <v>0.1668</v>
       </c>
       <c r="G31">
-        <v>0.4658</v>
+        <v>0.4639</v>
       </c>
       <c r="H31">
         <v>0.8445</v>
@@ -1189,16 +1189,16 @@
         <v>27.6</v>
       </c>
       <c r="D32">
-        <v>0.3029</v>
+        <v>0.3022</v>
       </c>
       <c r="E32">
-        <v>0.3017</v>
+        <v>0.302</v>
       </c>
       <c r="F32">
         <v>0.3021</v>
       </c>
       <c r="G32">
-        <v>0.4778</v>
+        <v>0.4768</v>
       </c>
       <c r="H32">
         <v>0.8905999999999999</v>
@@ -1215,16 +1215,16 @@
         <v>25.8</v>
       </c>
       <c r="D33">
-        <v>0.2057</v>
+        <v>0.2051</v>
       </c>
       <c r="E33">
-        <v>0.2047</v>
+        <v>0.205</v>
       </c>
       <c r="F33">
         <v>0.205</v>
       </c>
       <c r="G33">
-        <v>0.4828</v>
+        <v>0.4814</v>
       </c>
       <c r="H33">
         <v>0.8759</v>
@@ -1241,16 +1241,16 @@
         <v>27.4</v>
       </c>
       <c r="D34">
-        <v>0.2753</v>
+        <v>0.2747</v>
       </c>
       <c r="E34">
-        <v>0.2742</v>
+        <v>0.2745</v>
       </c>
       <c r="F34">
         <v>0.2746</v>
       </c>
       <c r="G34">
-        <v>0.4698</v>
+        <v>0.4688</v>
       </c>
       <c r="H34">
         <v>0.8759</v>
@@ -1267,16 +1267,16 @@
         <v>25.8</v>
       </c>
       <c r="D35">
-        <v>0.199</v>
+        <v>0.1984</v>
       </c>
       <c r="E35">
-        <v>0.1979</v>
+        <v>0.1983</v>
       </c>
       <c r="F35">
         <v>0.1983</v>
       </c>
       <c r="G35">
-        <v>0.4678</v>
+        <v>0.4662</v>
       </c>
       <c r="H35">
         <v>0.8854</v>
@@ -1293,16 +1293,16 @@
         <v>21.8</v>
       </c>
       <c r="D36">
-        <v>0.1152</v>
+        <v>0.1144</v>
       </c>
       <c r="E36">
-        <v>0.1138</v>
+        <v>0.1142</v>
       </c>
       <c r="F36">
         <v>0.1143</v>
       </c>
       <c r="G36">
-        <v>0.4106</v>
+        <v>0.4077</v>
       </c>
       <c r="H36">
         <v>0.7655</v>
@@ -1319,16 +1319,16 @@
         <v>22.9</v>
       </c>
       <c r="D37">
-        <v>0.1322</v>
+        <v>0.1316</v>
       </c>
       <c r="E37">
-        <v>0.1312</v>
+        <v>0.1315</v>
       </c>
       <c r="F37">
         <v>0.1315</v>
       </c>
       <c r="G37">
-        <v>0.5344</v>
+        <v>0.5317</v>
       </c>
       <c r="H37">
         <v>0.9226</v>

</xml_diff>